<commit_message>
Corrida | GSF-EPUB | 2026-05-07 12:45:45.349013
</commit_message>
<xml_diff>
--- a/indicadores/GSF-EPUB_out.xlsx
+++ b/indicadores/GSF-EPUB_out.xlsx
@@ -6720,4 +6720,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECDC6ACE-C0A2-43B8-AE2D-64130EE5F484}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F44FE9A6-F6BD-4A06-9DEC-297FF880177E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C22993D0-D0CE-43CC-BA7D-1EB11030C5A8}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | GSF-EPUB | 2026-05-07 13:06:42.13632
</commit_message>
<xml_diff>
--- a/indicadores/GSF-EPUB_out.xlsx
+++ b/indicadores/GSF-EPUB_out.xlsx
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">vcorvalan</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -6944,13 +6944,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECDC6ACE-C0A2-43B8-AE2D-64130EE5F484}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F0E3F6F-DDC6-4ABF-B73D-38F14947BDBA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F44FE9A6-F6BD-4A06-9DEC-297FF880177E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7FC476B-62D8-4B68-8015-057B88579772}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C22993D0-D0CE-43CC-BA7D-1EB11030C5A8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B7FA95A-549A-4098-91BC-39EC262178B4}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | GSF-EPUB | 2026-06-17 11:35:01.811146
</commit_message>
<xml_diff>
--- a/indicadores/GSF-EPUB_out.xlsx
+++ b/indicadores/GSF-EPUB_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="179">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Ocupados en el sector público del Gran Santa Fe</t>
+    <t xml:space="preserve">Ocupados en el sector público</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aglomerado Gran Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1047,9 +1053,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1060,7 +1070,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1074,12 +1084,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.275871470742881</v>
+        <v>0.268324339798877</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1090,7 +1100,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1118,7 +1128,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1132,12 +1142,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0223792843976097</v>
+        <v>0.0251878407593091</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1160,7 +1170,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1174,7 +1184,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1188,7 +1198,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1202,12 +1212,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00704157508379751</v>
+        <v>0.00872811059952</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1218,7 +1228,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1232,12 +1242,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.79818838924137</v>
+        <v>0.874084652090649</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1380,10 +1390,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1396,10 +1406,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1423,66 +1433,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>40.382</v>
@@ -1535,7 +1545,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>39.128</v>
@@ -1592,7 +1602,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>41.255</v>
@@ -1649,7 +1659,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>38.135</v>
@@ -1706,7 +1716,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>39.451</v>
@@ -1765,7 +1775,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>36.088</v>
@@ -1824,7 +1834,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>35.364</v>
@@ -1883,7 +1893,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>38.249</v>
@@ -1942,7 +1952,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>35.512</v>
@@ -2001,7 +2011,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>42.694</v>
@@ -2060,7 +2070,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>43.215</v>
@@ -2119,7 +2129,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>38.854</v>
@@ -2178,7 +2188,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>44.001</v>
@@ -2237,7 +2247,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>44.777</v>
@@ -2296,7 +2306,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>43.288</v>
@@ -2355,7 +2365,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>42.023</v>
@@ -2414,7 +2424,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>48.478</v>
@@ -2473,7 +2483,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>51.223</v>
@@ -2532,7 +2542,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>42.247</v>
@@ -2591,7 +2601,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>46.849</v>
@@ -2650,7 +2660,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>58.259</v>
@@ -2709,7 +2719,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>53.977</v>
@@ -2768,7 +2778,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>47.06</v>
@@ -2827,7 +2837,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>49.032</v>
@@ -2886,7 +2896,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>54.016</v>
@@ -2945,7 +2955,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>51.252</v>
@@ -3004,7 +3014,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>48.855</v>
@@ -3063,7 +3073,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>46.384</v>
@@ -3122,7 +3132,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>48.182</v>
@@ -3181,7 +3191,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>42.801</v>
@@ -3240,7 +3250,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>41.173</v>
@@ -3299,7 +3309,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>46.762</v>
@@ -3358,7 +3368,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>49.253</v>
@@ -3417,7 +3427,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>43.98</v>
@@ -3476,7 +3486,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>42.412</v>
@@ -3535,7 +3545,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>50.32</v>
@@ -3594,7 +3604,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>52.582</v>
@@ -3653,7 +3663,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>44.65</v>
@@ -3712,7 +3722,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>43.651</v>
@@ -3771,7 +3781,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>53.878</v>
@@ -3830,7 +3840,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>55.911</v>
@@ -3889,7 +3899,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>47.518</v>
@@ -3948,7 +3958,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>48.053</v>
@@ -4007,7 +4017,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>52.985</v>
@@ -4066,7 +4076,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>53.805</v>
@@ -4125,7 +4135,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>51.089</v>
@@ -4184,7 +4194,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>53.311</v>
@@ -4243,7 +4253,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>57.045</v>
@@ -4302,7 +4312,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>58.277</v>
@@ -4361,7 +4371,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>51.191</v>
@@ -4420,7 +4430,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>56.535</v>
@@ -4479,7 +4489,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>62.113</v>
@@ -4538,7 +4548,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>53.27</v>
@@ -4597,7 +4607,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>48.455</v>
@@ -4656,7 +4666,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>49.068</v>
@@ -4715,7 +4725,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>53.828</v>
@@ -4774,7 +4784,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>49.391</v>
@@ -4833,7 +4843,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>49.029</v>
@@ -4892,7 +4902,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>54.484</v>
@@ -4951,7 +4961,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>58.759</v>
@@ -5010,7 +5020,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>51.099</v>
@@ -5069,7 +5079,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>48.786</v>
@@ -5128,7 +5138,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>58.929</v>
@@ -5187,7 +5197,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>51.654</v>
@@ -5246,7 +5256,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>41.524</v>
@@ -5305,7 +5315,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>43.751</v>
@@ -5364,7 +5374,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>46.819</v>
@@ -5423,7 +5433,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>45.535</v>
@@ -5482,7 +5492,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>42.418</v>
@@ -5541,7 +5551,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>48.256</v>
@@ -5600,7 +5610,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>46.223</v>
@@ -5659,7 +5669,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>49.692</v>
@@ -5718,7 +5728,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>51.943</v>
@@ -5777,7 +5787,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>55.609</v>
@@ -5836,7 +5846,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>44.919</v>
@@ -5895,7 +5905,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>43.842</v>
@@ -5954,7 +5964,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2"/>
       <c r="C78" s="3" t="n">
@@ -5987,7 +5997,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2"/>
       <c r="C79" s="3" t="n">
@@ -6020,7 +6030,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2"/>
       <c r="C80" s="3" t="n">
@@ -6053,7 +6063,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2"/>
       <c r="C81" s="3" t="n">
@@ -6086,7 +6096,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2"/>
       <c r="C82" s="3"/>
@@ -6109,7 +6119,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
@@ -6132,7 +6142,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2"/>
       <c r="C84" s="3"/>
@@ -6155,7 +6165,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2"/>
       <c r="C85" s="3"/>
@@ -6178,7 +6188,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2"/>
       <c r="C86" s="3"/>
@@ -6201,7 +6211,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2"/>
       <c r="C87" s="3"/>
@@ -6224,7 +6234,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2"/>
       <c r="C88" s="3"/>
@@ -6247,7 +6257,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2"/>
       <c r="C89" s="3"/>
@@ -6270,7 +6280,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2"/>
       <c r="C90" s="3"/>
@@ -6293,7 +6303,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2"/>
       <c r="C91" s="3"/>
@@ -6316,7 +6326,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2"/>
       <c r="C92" s="3"/>
@@ -6339,7 +6349,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2"/>
       <c r="C93" s="3"/>
@@ -6362,7 +6372,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2"/>
       <c r="C94" s="3"/>
@@ -6385,7 +6395,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2"/>
       <c r="C95" s="3"/>
@@ -6408,7 +6418,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
@@ -6431,7 +6441,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="3"/>
@@ -6465,97 +6475,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -6579,7 +6589,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -6589,80 +6599,80 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.275871470742881</v>
+        <v>0.268324339798877</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0970950569594505</v>
+        <v>0.0923100736222232</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.0946392673146209</v>
+        <v>-0.0904329959563043</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>-0.0307821719066232</v>
+        <v>-0.021206475320898</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.149597073492798</v>
+        <v>0.158706776034639</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.1656656969087</v>
+        <v>0.165413094411826</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>-0.0149014000970461</v>
+        <v>-0.0237510641572777</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.206697253603492</v>
+        <v>-0.208647825294298</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.186360528193574</v>
+        <v>-0.178440807103116</v>
       </c>
     </row>
     <row r="14">
@@ -6720,237 +6730,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F0E3F6F-DDC6-4ABF-B73D-38F14947BDBA}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7FC476B-62D8-4B68-8015-057B88579772}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B7FA95A-549A-4098-91BC-39EC262178B4}"/>
 </file>
</xml_diff>